<commit_message>
Created some educactional SPICE sims
</commit_message>
<xml_diff>
--- a/Flyback_Converter/Demo_Flyback_Converter_Design_Calculations.xlsx
+++ b/Flyback_Converter/Demo_Flyback_Converter_Design_Calculations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vvuon\Documents\KiCad_Projects\Flyback_Converter_Demo_Board\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vvuon\Documents\LTspice_Projects\Flyback_Converter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBCF1A86-6145-458D-B8E7-A43240E4FFEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36206666-105B-4B59-B61F-68D35A37FEE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21820" xr2:uid="{2ABFD8E1-7393-41CC-8605-39C70B410F57}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="21690" xr2:uid="{2ABFD8E1-7393-41CC-8605-39C70B410F57}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -548,7 +548,7 @@
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="H3" s="2">
-        <v>1.0000000000000001E-5</v>
+        <v>4.1999999999999998E-5</v>
       </c>
       <c r="I3" s="1">
         <v>0.05</v>
@@ -603,6 +603,7 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
+        <f>$A$3</f>
         <v>5</v>
       </c>
       <c r="B7" s="1">
@@ -614,7 +615,7 @@
       </c>
       <c r="D7" s="2">
         <f>$H$3</f>
-        <v>1.0000000000000001E-5</v>
+        <v>4.1999999999999998E-5</v>
       </c>
       <c r="E7" s="2">
         <f>$F$3</f>
@@ -626,23 +627,24 @@
       </c>
       <c r="G7" s="2">
         <f>(A7/B7)/SQRT((C7*F7)/(2*D7))</f>
-        <v>3.5355339059327376E-2</v>
+        <v>7.2456883730947191E-2</v>
       </c>
       <c r="H7" s="2">
         <f>G7*$G$3</f>
-        <v>3.5355339059327379E-7</v>
+        <v>7.2456883730947201E-7</v>
       </c>
       <c r="I7" s="2">
         <f>$G$3-H7</f>
-        <v>9.6464466094067262E-6</v>
+        <v>9.2754311626905287E-6</v>
       </c>
       <c r="J7" s="2">
         <f>($C$3*I7)/($I$3)</f>
-        <v>3.8585786437626905E-4</v>
+        <v>3.7101724650762113E-4</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
+        <f>$A$3</f>
         <v>5</v>
       </c>
       <c r="B8" s="1">
@@ -654,7 +656,7 @@
       </c>
       <c r="D8" s="2">
         <f>$H$3</f>
-        <v>1.0000000000000001E-5</v>
+        <v>4.1999999999999998E-5</v>
       </c>
       <c r="E8" s="2">
         <f>$F$3</f>
@@ -666,19 +668,19 @@
       </c>
       <c r="G8" s="2">
         <f>(A8/B8)/SQRT((C8*F8)/(2*D8))</f>
-        <v>1.7677669529663688E-2</v>
+        <v>3.6228441865473596E-2</v>
       </c>
       <c r="H8" s="2">
         <f>G8*$G$3</f>
-        <v>1.7677669529663689E-7</v>
+        <v>3.62284418654736E-7</v>
       </c>
       <c r="I8" s="2">
         <f>$G$3-H8</f>
-        <v>9.8232233047033644E-6</v>
+        <v>9.6377155813452648E-6</v>
       </c>
       <c r="J8" s="2">
         <f>($C$3*I8)/($I$3)</f>
-        <v>3.9292893218813453E-4</v>
+        <v>3.8550862325381055E-4</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
@@ -729,6 +731,7 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
+        <f>$A$3</f>
         <v>5</v>
       </c>
       <c r="B14" s="1">
@@ -740,7 +743,7 @@
       </c>
       <c r="D14" s="2">
         <f>$H$3</f>
-        <v>1.0000000000000001E-5</v>
+        <v>4.1999999999999998E-5</v>
       </c>
       <c r="E14" s="2">
         <f>$F$3</f>
@@ -752,27 +755,28 @@
       </c>
       <c r="G14" s="2">
         <f>(A14/B14)/SQRT((C14*F14)/(2*D14))</f>
-        <v>0.22360679774997896</v>
+        <v>0.45825756949558394</v>
       </c>
       <c r="H14" s="2">
         <f>G14*$G$3</f>
-        <v>2.2360679774997899E-6</v>
+        <v>4.5825756949558395E-6</v>
       </c>
       <c r="I14" s="2">
         <f>$G$3-H14</f>
-        <v>7.76393202250021E-6</v>
+        <v>5.4174243050441613E-6</v>
       </c>
       <c r="J14" s="2">
         <f>($C$3*I14)/($I$3)</f>
-        <v>3.1055728090000837E-4</v>
+        <v>2.1669697220176644E-4</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
+        <f>$A$3</f>
         <v>5</v>
       </c>
       <c r="B15" s="1">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C15" s="1">
         <f>$E$3</f>
@@ -780,7 +784,7 @@
       </c>
       <c r="D15" s="2">
         <f>$H$3</f>
-        <v>1.0000000000000001E-5</v>
+        <v>4.1999999999999998E-5</v>
       </c>
       <c r="E15" s="2">
         <f>$F$3</f>
@@ -792,19 +796,19 @@
       </c>
       <c r="G15" s="2">
         <f>(A15/B15)/SQRT((C15*F15)/(2*D15))</f>
-        <v>0.13153341044116409</v>
+        <v>0.22912878474779197</v>
       </c>
       <c r="H15" s="2">
         <f>G15*$G$3</f>
-        <v>1.315334104411641E-6</v>
+        <v>2.2912878474779198E-6</v>
       </c>
       <c r="I15" s="2">
         <f>$G$3-H15</f>
-        <v>8.6846658955883598E-6</v>
+        <v>7.7087121525220811E-6</v>
       </c>
       <c r="J15" s="2">
         <f>($C$3*I15)/($I$3)</f>
-        <v>3.4738663582353438E-4</v>
+        <v>3.0834848610088324E-4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Started a bunch of new projects
</commit_message>
<xml_diff>
--- a/Flyback_Converter/Demo_Flyback_Converter_Design_Calculations.xlsx
+++ b/Flyback_Converter/Demo_Flyback_Converter_Design_Calculations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vvuon\Documents\LTspice_Projects\Flyback_Converter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36206666-105B-4B59-B61F-68D35A37FEE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F748040-B831-45E0-BE1C-AC5B111F358D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="21690" xr2:uid="{2ABFD8E1-7393-41CC-8605-39C70B410F57}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{2ABFD8E1-7393-41CC-8605-39C70B410F57}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="20">
   <si>
     <t>VOUT</t>
   </si>
@@ -93,6 +93,12 @@
   </si>
   <si>
     <t>VOUT (V)</t>
+  </si>
+  <si>
+    <t>VIN_MIN (V)</t>
+  </si>
+  <si>
+    <t>VIN_MAX (V)</t>
   </si>
 </sst>
 </file>
@@ -484,78 +490,93 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3535560F-19EB-4294-B8E4-B82D051408B5}">
-  <dimension ref="A2:J15"/>
+  <dimension ref="A2:K15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.6328125" customWidth="1"/>
+    <col min="2" max="2" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7265625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.7265625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.81640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="34.81640625" customWidth="1"/>
+    <col min="11" max="11" width="10.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>5</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="1">
+        <v>20</v>
+      </c>
+      <c r="C3" s="1">
+        <v>40</v>
+      </c>
+      <c r="D3" s="2">
         <v>0.05</v>
       </c>
-      <c r="C3" s="1">
+      <c r="E3" s="1">
         <v>2</v>
       </c>
-      <c r="D3" s="2">
-        <f>A3/B3</f>
+      <c r="F3" s="2">
+        <f>A3/D3</f>
         <v>100</v>
       </c>
-      <c r="E3" s="1">
-        <f>A3/C3</f>
+      <c r="G3" s="1">
+        <f>A3/E3</f>
         <v>2.5</v>
       </c>
-      <c r="F3" s="2">
+      <c r="H3" s="2">
         <v>100000</v>
       </c>
-      <c r="G3" s="2">
-        <f>1/F3</f>
-        <v>1.0000000000000001E-5</v>
-      </c>
-      <c r="H3" s="2">
-        <v>4.1999999999999998E-5</v>
-      </c>
-      <c r="I3" s="1">
+      <c r="I3" s="2">
+        <f>1/H3</f>
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="J3" s="2">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="K3" s="1">
         <v>0.05</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>11</v>
       </c>
@@ -569,7 +590,7 @@
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -601,89 +622,91 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <f>$A$3</f>
         <v>5</v>
       </c>
       <c r="B7" s="1">
+        <f>$B$3</f>
         <v>20</v>
       </c>
       <c r="C7" s="2">
-        <f>$D$3</f>
+        <f>$F$3</f>
         <v>100</v>
       </c>
       <c r="D7" s="2">
+        <f>$J$3</f>
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="E7" s="2">
         <f>$H$3</f>
-        <v>4.1999999999999998E-5</v>
-      </c>
-      <c r="E7" s="2">
-        <f>$F$3</f>
         <v>100000</v>
       </c>
       <c r="F7" s="2">
-        <f>$G$3</f>
+        <f>$I$3</f>
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="G7" s="2">
         <f>(A7/B7)/SQRT((C7*F7)/(2*D7))</f>
-        <v>7.2456883730947191E-2</v>
+        <v>3.5355339059327376E-2</v>
       </c>
       <c r="H7" s="2">
-        <f>G7*$G$3</f>
-        <v>7.2456883730947201E-7</v>
+        <f>G7*$I$3</f>
+        <v>3.5355339059327379E-7</v>
       </c>
       <c r="I7" s="2">
-        <f>$G$3-H7</f>
-        <v>9.2754311626905287E-6</v>
+        <f>$I$3-H7</f>
+        <v>9.6464466094067262E-6</v>
       </c>
       <c r="J7" s="2">
-        <f>($C$3*I7)/($I$3)</f>
-        <v>3.7101724650762113E-4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+        <f>($E$3*I7)/($K$3)</f>
+        <v>3.8585786437626905E-4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <f>$A$3</f>
         <v>5</v>
       </c>
       <c r="B8" s="1">
+        <f>$C$3</f>
         <v>40</v>
       </c>
       <c r="C8" s="2">
-        <f>$D$3</f>
+        <f>$F$3</f>
         <v>100</v>
       </c>
       <c r="D8" s="2">
+        <f>$J$3</f>
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="E8" s="2">
         <f>$H$3</f>
-        <v>4.1999999999999998E-5</v>
-      </c>
-      <c r="E8" s="2">
-        <f>$F$3</f>
         <v>100000</v>
       </c>
       <c r="F8" s="2">
-        <f>$G$3</f>
+        <f>$I$3</f>
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="G8" s="2">
         <f>(A8/B8)/SQRT((C8*F8)/(2*D8))</f>
-        <v>3.6228441865473596E-2</v>
+        <v>1.7677669529663688E-2</v>
       </c>
       <c r="H8" s="2">
-        <f>G8*$G$3</f>
-        <v>3.62284418654736E-7</v>
+        <f>G8*$I$3</f>
+        <v>1.7677669529663689E-7</v>
       </c>
       <c r="I8" s="2">
-        <f>$G$3-H8</f>
-        <v>9.6377155813452648E-6</v>
+        <f>$I$3-H8</f>
+        <v>9.8232233047033644E-6</v>
       </c>
       <c r="J8" s="2">
-        <f>($C$3*I8)/($I$3)</f>
-        <v>3.8550862325381055E-4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+        <f>($E$3*I8)/($K$3)</f>
+        <v>3.9292893218813453E-4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>12</v>
       </c>
@@ -697,7 +720,7 @@
       <c r="I12" s="3"/>
       <c r="J12" s="3"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>0</v>
       </c>
@@ -729,86 +752,88 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <f>$A$3</f>
         <v>5</v>
       </c>
       <c r="B14" s="1">
+        <f>$B$3</f>
         <v>20</v>
       </c>
       <c r="C14" s="1">
-        <f>$E$3</f>
+        <f>$G$3</f>
         <v>2.5</v>
       </c>
       <c r="D14" s="2">
+        <f>$J$3</f>
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="E14" s="2">
         <f>$H$3</f>
-        <v>4.1999999999999998E-5</v>
-      </c>
-      <c r="E14" s="2">
-        <f>$F$3</f>
         <v>100000</v>
       </c>
       <c r="F14" s="2">
-        <f>$G$3</f>
+        <f>$I$3</f>
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="G14" s="2">
         <f>(A14/B14)/SQRT((C14*F14)/(2*D14))</f>
-        <v>0.45825756949558394</v>
+        <v>0.22360679774997896</v>
       </c>
       <c r="H14" s="2">
-        <f>G14*$G$3</f>
-        <v>4.5825756949558395E-6</v>
+        <f>G14*$I$3</f>
+        <v>2.2360679774997899E-6</v>
       </c>
       <c r="I14" s="2">
-        <f>$G$3-H14</f>
-        <v>5.4174243050441613E-6</v>
+        <f>$I$3-H14</f>
+        <v>7.76393202250021E-6</v>
       </c>
       <c r="J14" s="2">
-        <f>($C$3*I14)/($I$3)</f>
-        <v>2.1669697220176644E-4</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+        <f>($E$3*I14)/($K$3)</f>
+        <v>3.1055728090000837E-4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <f>$A$3</f>
         <v>5</v>
       </c>
       <c r="B15" s="1">
+        <f>$C$3</f>
         <v>40</v>
       </c>
       <c r="C15" s="1">
-        <f>$E$3</f>
+        <f>$G$3</f>
         <v>2.5</v>
       </c>
       <c r="D15" s="2">
+        <f>$J$3</f>
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="E15" s="2">
         <f>$H$3</f>
-        <v>4.1999999999999998E-5</v>
-      </c>
-      <c r="E15" s="2">
-        <f>$F$3</f>
         <v>100000</v>
       </c>
       <c r="F15" s="2">
-        <f>$G$3</f>
+        <f>$I$3</f>
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="G15" s="2">
         <f>(A15/B15)/SQRT((C15*F15)/(2*D15))</f>
-        <v>0.22912878474779197</v>
+        <v>0.11180339887498948</v>
       </c>
       <c r="H15" s="2">
-        <f>G15*$G$3</f>
-        <v>2.2912878474779198E-6</v>
+        <f>G15*$I$3</f>
+        <v>1.118033988749895E-6</v>
       </c>
       <c r="I15" s="2">
-        <f>$G$3-H15</f>
-        <v>7.7087121525220811E-6</v>
+        <f>$I$3-H15</f>
+        <v>8.8819660112501063E-6</v>
       </c>
       <c r="J15" s="2">
-        <f>($C$3*I15)/($I$3)</f>
-        <v>3.0834848610088324E-4</v>
+        <f>($E$3*I15)/($K$3)</f>
+        <v>3.5527864045000422E-4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>